<commit_message>
Split commit 1 (final batch)
</commit_message>
<xml_diff>
--- a/writerConference/rssi_output.xlsx
+++ b/writerConference/rssi_output.xlsx
@@ -2841,2410 +2841,2410 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>-29.54437828063965</v>
+        <v>-31.73988914489746</v>
       </c>
       <c r="B1" t="n">
-        <v>-35.09778213500977</v>
+        <v>-32.42946243286133</v>
       </c>
       <c r="C1" t="n">
-        <v>-41.01274871826172</v>
+        <v>-35.58815383911133</v>
       </c>
       <c r="D1" t="n">
-        <v>-42.41579055786133</v>
+        <v>-36.15460968017578</v>
       </c>
       <c r="E1" t="n">
-        <v>-46.1126823425293</v>
+        <v>-40.74419403076172</v>
       </c>
       <c r="F1" t="n">
-        <v>-52.49204635620117</v>
+        <v>-39.8609733581543</v>
       </c>
       <c r="G1" t="n">
-        <v>-62.20493316650391</v>
+        <v>-42.57514190673828</v>
       </c>
       <c r="H1" t="n">
-        <v>-57.30550384521484</v>
+        <v>-46.60338592529297</v>
       </c>
       <c r="I1" t="n">
-        <v>-57.74993896484375</v>
+        <v>-48.25447463989258</v>
       </c>
       <c r="J1" t="n">
-        <v>-63.20989990234375</v>
+        <v>-44.60097503662109</v>
       </c>
       <c r="K1" t="n">
-        <v>-60.74666213989258</v>
+        <v>-44.7952995300293</v>
       </c>
       <c r="L1" t="n">
-        <v>-60.6839714050293</v>
+        <v>-45.5946044921875</v>
       </c>
       <c r="M1" t="n">
-        <v>-60.12469482421875</v>
+        <v>-50.12831878662109</v>
       </c>
       <c r="N1" t="n">
-        <v>-63.78755950927734</v>
+        <v>-50.54061126708984</v>
       </c>
       <c r="O1" t="n">
-        <v>-63.51335525512695</v>
+        <v>-50.35604858398438</v>
       </c>
       <c r="P1" t="n">
-        <v>-68.05302429199219</v>
+        <v>-51.69874954223633</v>
       </c>
       <c r="Q1" t="n">
-        <v>-69.68775939941406</v>
+        <v>-50.63460159301758</v>
       </c>
       <c r="R1" t="n">
-        <v>-77.74272155761719</v>
+        <v>-52.20363616943359</v>
       </c>
       <c r="S1" t="n">
-        <v>-68.48191070556641</v>
+        <v>-54.53389739990234</v>
       </c>
       <c r="T1" t="n">
-        <v>-68.33390808105469</v>
+        <v>-52.3571662902832</v>
       </c>
       <c r="U1" t="n">
-        <v>-73.78950500488281</v>
+        <v>-51.42533111572266</v>
       </c>
       <c r="V1" t="n">
-        <v>-77.72330474853516</v>
+        <v>-52.77375411987305</v>
       </c>
       <c r="W1" t="n">
-        <v>-69.94468688964844</v>
+        <v>-52.99045562744141</v>
       </c>
       <c r="X1" t="n">
-        <v>-75.05682373046875</v>
+        <v>-56.56414031982422</v>
       </c>
       <c r="Y1" t="n">
-        <v>-76.90386199951172</v>
+        <v>-57.21269989013672</v>
       </c>
       <c r="Z1" t="n">
-        <v>-75.89933776855469</v>
+        <v>-57.63677978515625</v>
       </c>
       <c r="AA1" t="n">
-        <v>-75.65846252441406</v>
+        <v>-57.56461715698242</v>
       </c>
       <c r="AB1" t="n">
-        <v>-75.3387451171875</v>
+        <v>-60.49135589599609</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>-36.37484359741211</v>
+        <v>-36.81267929077148</v>
       </c>
       <c r="B2" t="n">
-        <v>-38.46696090698242</v>
+        <v>-34.91189575195312</v>
       </c>
       <c r="C2" t="n">
-        <v>-44.7988166809082</v>
+        <v>-38.66301727294922</v>
       </c>
       <c r="D2" t="n">
-        <v>-50.35476303100586</v>
+        <v>-40.37996292114258</v>
       </c>
       <c r="E2" t="n">
-        <v>-48.74587249755859</v>
+        <v>-42.16316986083984</v>
       </c>
       <c r="F2" t="n">
-        <v>-53.66500091552734</v>
+        <v>-41.91585922241211</v>
       </c>
       <c r="G2" t="n">
-        <v>-53.6481819152832</v>
+        <v>-40.94680023193359</v>
       </c>
       <c r="H2" t="n">
-        <v>-59.8607177734375</v>
+        <v>-46.98404693603516</v>
       </c>
       <c r="I2" t="n">
-        <v>-51.56760406494141</v>
+        <v>-45.71127700805664</v>
       </c>
       <c r="J2" t="n">
-        <v>-55.54486083984375</v>
+        <v>-44.61403656005859</v>
       </c>
       <c r="K2" t="n">
-        <v>-58.60979461669922</v>
+        <v>-48.67433929443359</v>
       </c>
       <c r="L2" t="n">
-        <v>-63.21550750732422</v>
+        <v>-51.93740844726562</v>
       </c>
       <c r="M2" t="n">
-        <v>-65.6240234375</v>
+        <v>-49.50347137451172</v>
       </c>
       <c r="N2" t="n">
-        <v>-64.44802093505859</v>
+        <v>-48.62194442749023</v>
       </c>
       <c r="O2" t="n">
-        <v>-70.02189636230469</v>
+        <v>-51.27848052978516</v>
       </c>
       <c r="P2" t="n">
-        <v>-68.05671691894531</v>
+        <v>-49.85099411010742</v>
       </c>
       <c r="Q2" t="n">
-        <v>-71.44490051269531</v>
+        <v>-50.41632843017578</v>
       </c>
       <c r="R2" t="n">
-        <v>-64.06539154052734</v>
+        <v>-51.35309600830078</v>
       </c>
       <c r="S2" t="n">
-        <v>-71.24034118652344</v>
+        <v>-52.60859298706055</v>
       </c>
       <c r="T2" t="n">
-        <v>-72.27819061279297</v>
+        <v>-49.4244270324707</v>
       </c>
       <c r="U2" t="n">
-        <v>-75.3365478515625</v>
+        <v>-51.58549880981445</v>
       </c>
       <c r="V2" t="n">
-        <v>-73.19606018066406</v>
+        <v>-53.13056182861328</v>
       </c>
       <c r="W2" t="n">
-        <v>-75.32147216796875</v>
+        <v>-52.93049240112305</v>
       </c>
       <c r="X2" t="n">
-        <v>-74.86286926269531</v>
+        <v>-52.4065055847168</v>
       </c>
       <c r="Y2" t="n">
-        <v>-78.84580993652344</v>
+        <v>-54.28730392456055</v>
       </c>
       <c r="Z2" t="n">
-        <v>-77.59410858154297</v>
+        <v>-53.90579986572266</v>
       </c>
       <c r="AA2" t="n">
-        <v>-75.27999114990234</v>
+        <v>-53.74308395385742</v>
       </c>
       <c r="AB2" t="n">
-        <v>-72.82197570800781</v>
+        <v>-56.30080032348633</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>-43.41970062255859</v>
+        <v>-38.54506683349609</v>
       </c>
       <c r="B3" t="n">
-        <v>-41.01880645751953</v>
+        <v>-37.9269905090332</v>
       </c>
       <c r="C3" t="n">
-        <v>-42.00269317626953</v>
+        <v>-38.3278923034668</v>
       </c>
       <c r="D3" t="n">
-        <v>-48.01739883422852</v>
+        <v>-42.82613754272461</v>
       </c>
       <c r="E3" t="n">
-        <v>-50.64441680908203</v>
+        <v>-44.05791091918945</v>
       </c>
       <c r="F3" t="n">
-        <v>-53.39120483398438</v>
+        <v>-42.48711013793945</v>
       </c>
       <c r="G3" t="n">
-        <v>-58.32489776611328</v>
+        <v>-47.54775619506836</v>
       </c>
       <c r="H3" t="n">
-        <v>-52.07361602783203</v>
+        <v>-42.41589736938477</v>
       </c>
       <c r="I3" t="n">
-        <v>-55.20713043212891</v>
+        <v>-46.82323455810547</v>
       </c>
       <c r="J3" t="n">
-        <v>-57.81122970581055</v>
+        <v>-43.73761749267578</v>
       </c>
       <c r="K3" t="n">
-        <v>-59.76673126220703</v>
+        <v>-46.90348434448242</v>
       </c>
       <c r="L3" t="n">
-        <v>-67.95746612548828</v>
+        <v>-48.34639739990234</v>
       </c>
       <c r="M3" t="n">
-        <v>-59.70587158203125</v>
+        <v>-50.9393196105957</v>
       </c>
       <c r="N3" t="n">
-        <v>-68.75422668457031</v>
+        <v>-48.37625885009766</v>
       </c>
       <c r="O3" t="n">
-        <v>-72.50413513183594</v>
+        <v>-49.11184310913086</v>
       </c>
       <c r="P3" t="n">
-        <v>-68.45909881591797</v>
+        <v>-50.50649261474609</v>
       </c>
       <c r="Q3" t="n">
-        <v>-63.7124137878418</v>
+        <v>-52.43607330322266</v>
       </c>
       <c r="R3" t="n">
-        <v>-73.39876556396484</v>
+        <v>-51.2906608581543</v>
       </c>
       <c r="S3" t="n">
-        <v>-67.73902893066406</v>
+        <v>-55.76071166992188</v>
       </c>
       <c r="T3" t="n">
-        <v>-69.25592041015625</v>
+        <v>-50.20852661132812</v>
       </c>
       <c r="U3" t="n">
-        <v>-74.91688537597656</v>
+        <v>-55.50812530517578</v>
       </c>
       <c r="V3" t="n">
-        <v>-73.96766662597656</v>
+        <v>-51.6044807434082</v>
       </c>
       <c r="W3" t="n">
-        <v>-75.2691650390625</v>
+        <v>-53.99892044067383</v>
       </c>
       <c r="X3" t="n">
-        <v>-74.10276794433594</v>
+        <v>-53.87089920043945</v>
       </c>
       <c r="Y3" t="n">
-        <v>-76.21791839599609</v>
+        <v>-56.74726104736328</v>
       </c>
       <c r="Z3" t="n">
-        <v>-77.51340484619141</v>
+        <v>-54.44118118286133</v>
       </c>
       <c r="AA3" t="n">
-        <v>-75.91716766357422</v>
+        <v>-57.31298828125</v>
       </c>
       <c r="AB3" t="n">
-        <v>-81.95646667480469</v>
+        <v>-55.3466682434082</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>-42.06691741943359</v>
+        <v>-38.04422760009766</v>
       </c>
       <c r="B4" t="n">
-        <v>-45.3929328918457</v>
+        <v>-37.18502044677734</v>
       </c>
       <c r="C4" t="n">
-        <v>-47.88335418701172</v>
+        <v>-38.63078689575195</v>
       </c>
       <c r="D4" t="n">
-        <v>-48.65499114990234</v>
+        <v>-41.09058380126953</v>
       </c>
       <c r="E4" t="n">
-        <v>-51.37503814697266</v>
+        <v>-41.83008575439453</v>
       </c>
       <c r="F4" t="n">
-        <v>-55.06383514404297</v>
+        <v>-43.35531234741211</v>
       </c>
       <c r="G4" t="n">
-        <v>-53.37709808349609</v>
+        <v>-45.87278747558594</v>
       </c>
       <c r="H4" t="n">
-        <v>-56.39413452148438</v>
+        <v>-45.20355606079102</v>
       </c>
       <c r="I4" t="n">
-        <v>-54.93974685668945</v>
+        <v>-47.27805328369141</v>
       </c>
       <c r="J4" t="n">
-        <v>-58.98735427856445</v>
+        <v>-48.25748825073242</v>
       </c>
       <c r="K4" t="n">
-        <v>-62.66041946411133</v>
+        <v>-51.39498138427734</v>
       </c>
       <c r="L4" t="n">
-        <v>-59.360107421875</v>
+        <v>-48.55614471435547</v>
       </c>
       <c r="M4" t="n">
-        <v>-58.74775314331055</v>
+        <v>-48.38710403442383</v>
       </c>
       <c r="N4" t="n">
-        <v>-69.63628387451172</v>
+        <v>-47.0711669921875</v>
       </c>
       <c r="O4" t="n">
-        <v>-68.71076965332031</v>
+        <v>-50.01717376708984</v>
       </c>
       <c r="P4" t="n">
-        <v>-66.30245208740234</v>
+        <v>-51.92952728271484</v>
       </c>
       <c r="Q4" t="n">
-        <v>-74.60622406005859</v>
+        <v>-53.86928176879883</v>
       </c>
       <c r="R4" t="n">
-        <v>-65.97151184082031</v>
+        <v>-55.63983154296875</v>
       </c>
       <c r="S4" t="n">
-        <v>-71.87339782714844</v>
+        <v>-53.69623565673828</v>
       </c>
       <c r="T4" t="n">
-        <v>-71.088134765625</v>
+        <v>-52.71157073974609</v>
       </c>
       <c r="U4" t="n">
-        <v>-76.19334411621094</v>
+        <v>-50.58631134033203</v>
       </c>
       <c r="V4" t="n">
-        <v>-76.51402282714844</v>
+        <v>-54.9727897644043</v>
       </c>
       <c r="W4" t="n">
-        <v>-77.23451232910156</v>
+        <v>-54.3115348815918</v>
       </c>
       <c r="X4" t="n">
-        <v>-77.13478088378906</v>
+        <v>-56.59212112426758</v>
       </c>
       <c r="Y4" t="n">
-        <v>-75.2021484375</v>
+        <v>-54.1353874206543</v>
       </c>
       <c r="Z4" t="n">
-        <v>-74.92509460449219</v>
+        <v>-51.92157745361328</v>
       </c>
       <c r="AA4" t="n">
-        <v>-76.43038177490234</v>
+        <v>-55.03647613525391</v>
       </c>
       <c r="AB4" t="n">
-        <v>-75.56085968017578</v>
+        <v>-51.60871124267578</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>-50.16460418701172</v>
+        <v>-41.05666351318359</v>
       </c>
       <c r="B5" t="n">
-        <v>-46.64916610717773</v>
+        <v>-39.52852630615234</v>
       </c>
       <c r="C5" t="n">
-        <v>-55.9818229675293</v>
+        <v>-45.05177307128906</v>
       </c>
       <c r="D5" t="n">
-        <v>-58.77095413208008</v>
+        <v>-43.23124313354492</v>
       </c>
       <c r="E5" t="n">
-        <v>-53.42831420898438</v>
+        <v>-45.6072998046875</v>
       </c>
       <c r="F5" t="n">
-        <v>-57.83133697509766</v>
+        <v>-43.97835922241211</v>
       </c>
       <c r="G5" t="n">
-        <v>-60.41475296020508</v>
+        <v>-44.34788131713867</v>
       </c>
       <c r="H5" t="n">
-        <v>-58.34879684448242</v>
+        <v>-42.22414016723633</v>
       </c>
       <c r="I5" t="n">
-        <v>-58.86350250244141</v>
+        <v>-46.35562133789062</v>
       </c>
       <c r="J5" t="n">
-        <v>-68.05470275878906</v>
+        <v>-45.75962448120117</v>
       </c>
       <c r="K5" t="n">
-        <v>-62.17134475708008</v>
+        <v>-47.91632843017578</v>
       </c>
       <c r="L5" t="n">
-        <v>-65.17490386962891</v>
+        <v>-48.83633804321289</v>
       </c>
       <c r="M5" t="n">
-        <v>-64.36906433105469</v>
+        <v>-48.36687850952148</v>
       </c>
       <c r="N5" t="n">
-        <v>-69.65180206298828</v>
+        <v>-50.75573348999023</v>
       </c>
       <c r="O5" t="n">
-        <v>-64.45137023925781</v>
+        <v>-50.21101379394531</v>
       </c>
       <c r="P5" t="n">
-        <v>-69.39357757568359</v>
+        <v>-49.68480682373047</v>
       </c>
       <c r="Q5" t="n">
-        <v>-66.52571868896484</v>
+        <v>-50.76472473144531</v>
       </c>
       <c r="R5" t="n">
-        <v>-71.69207000732422</v>
+        <v>-53.2379264831543</v>
       </c>
       <c r="S5" t="n">
-        <v>-74.69950103759766</v>
+        <v>-54.4400520324707</v>
       </c>
       <c r="T5" t="n">
-        <v>-73.35207366943359</v>
+        <v>-52.08837127685547</v>
       </c>
       <c r="U5" t="n">
-        <v>-67.23939514160156</v>
+        <v>-52.79519653320312</v>
       </c>
       <c r="V5" t="n">
-        <v>-72.7122802734375</v>
+        <v>-54.89124298095703</v>
       </c>
       <c r="W5" t="n">
-        <v>-74.28065490722656</v>
+        <v>-52.30797576904297</v>
       </c>
       <c r="X5" t="n">
-        <v>-77.54673004150391</v>
+        <v>-53.9687385559082</v>
       </c>
       <c r="Y5" t="n">
-        <v>-72.62503814697266</v>
+        <v>-54.96966552734375</v>
       </c>
       <c r="Z5" t="n">
-        <v>-74.48170471191406</v>
+        <v>-59.09485626220703</v>
       </c>
       <c r="AA5" t="n">
-        <v>-78.1944580078125</v>
+        <v>-55.8912353515625</v>
       </c>
       <c r="AB5" t="n">
-        <v>-81.85810089111328</v>
+        <v>-52.83844757080078</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>-51.39049530029297</v>
+        <v>-40.99485015869141</v>
       </c>
       <c r="B6" t="n">
-        <v>-52.04323196411133</v>
+        <v>-44.61943054199219</v>
       </c>
       <c r="C6" t="n">
-        <v>-52.97794723510742</v>
+        <v>-40.77645111083984</v>
       </c>
       <c r="D6" t="n">
-        <v>-50.86052703857422</v>
+        <v>-44.27646636962891</v>
       </c>
       <c r="E6" t="n">
-        <v>-55.48836517333984</v>
+        <v>-43.09598922729492</v>
       </c>
       <c r="F6" t="n">
-        <v>-59.66237258911133</v>
+        <v>-43.15429306030273</v>
       </c>
       <c r="G6" t="n">
-        <v>-57.68551635742188</v>
+        <v>-45.61401748657227</v>
       </c>
       <c r="H6" t="n">
-        <v>-59.84402465820312</v>
+        <v>-46.14541244506836</v>
       </c>
       <c r="I6" t="n">
-        <v>-58.93107986450195</v>
+        <v>-44.73264312744141</v>
       </c>
       <c r="J6" t="n">
-        <v>-62.17662811279297</v>
+        <v>-50.25421905517578</v>
       </c>
       <c r="K6" t="n">
-        <v>-65.41178131103516</v>
+        <v>-45.63645172119141</v>
       </c>
       <c r="L6" t="n">
-        <v>-64.20021057128906</v>
+        <v>-48.66823959350586</v>
       </c>
       <c r="M6" t="n">
-        <v>-66.98896789550781</v>
+        <v>-52.6375732421875</v>
       </c>
       <c r="N6" t="n">
-        <v>-66.24797821044922</v>
+        <v>-52.8624267578125</v>
       </c>
       <c r="O6" t="n">
-        <v>-74.86843109130859</v>
+        <v>-50.93155288696289</v>
       </c>
       <c r="P6" t="n">
-        <v>-65.75113677978516</v>
+        <v>-49.86342620849609</v>
       </c>
       <c r="Q6" t="n">
-        <v>-69.96537017822266</v>
+        <v>-52.34780883789062</v>
       </c>
       <c r="R6" t="n">
-        <v>-75.50553894042969</v>
+        <v>-53.71743011474609</v>
       </c>
       <c r="S6" t="n">
-        <v>-66.23889923095703</v>
+        <v>-55.62947845458984</v>
       </c>
       <c r="T6" t="n">
-        <v>-71.11891937255859</v>
+        <v>-58.31301879882812</v>
       </c>
       <c r="U6" t="n">
-        <v>-71.88450622558594</v>
+        <v>-53.8682746887207</v>
       </c>
       <c r="V6" t="n">
-        <v>-79.20449829101562</v>
+        <v>-55.5026741027832</v>
       </c>
       <c r="W6" t="n">
-        <v>-80.64820098876953</v>
+        <v>-54.87021636962891</v>
       </c>
       <c r="X6" t="n">
-        <v>-77.52734375</v>
+        <v>-54.19746017456055</v>
       </c>
       <c r="Y6" t="n">
-        <v>-80.67929840087891</v>
+        <v>-51.78805541992188</v>
       </c>
       <c r="Z6" t="n">
-        <v>-72.54777526855469</v>
+        <v>-53.21662521362305</v>
       </c>
       <c r="AA6" t="n">
-        <v>-80.16984558105469</v>
+        <v>-54.3794059753418</v>
       </c>
       <c r="AB6" t="n">
-        <v>-85.80372619628906</v>
+        <v>-58.3748664855957</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>-52.26765060424805</v>
+        <v>-42.25920104980469</v>
       </c>
       <c r="B7" t="n">
-        <v>-57.50865936279297</v>
+        <v>-38.40400314331055</v>
       </c>
       <c r="C7" t="n">
-        <v>-53.4208984375</v>
+        <v>-40.46535873413086</v>
       </c>
       <c r="D7" t="n">
-        <v>-54.9112434387207</v>
+        <v>-46.57241821289062</v>
       </c>
       <c r="E7" t="n">
-        <v>-61.71776580810547</v>
+        <v>-42.15779876708984</v>
       </c>
       <c r="F7" t="n">
-        <v>-54.57615280151367</v>
+        <v>-44.89062881469727</v>
       </c>
       <c r="G7" t="n">
-        <v>-54.30014801025391</v>
+        <v>-47.35093307495117</v>
       </c>
       <c r="H7" t="n">
-        <v>-60.76111602783203</v>
+        <v>-46.50449752807617</v>
       </c>
       <c r="I7" t="n">
-        <v>-62.1512565612793</v>
+        <v>-45.70908737182617</v>
       </c>
       <c r="J7" t="n">
-        <v>-61.00127410888672</v>
+        <v>-47.87649154663086</v>
       </c>
       <c r="K7" t="n">
-        <v>-68.68573760986328</v>
+        <v>-48.74477767944336</v>
       </c>
       <c r="L7" t="n">
-        <v>-65.96830749511719</v>
+        <v>-45.71120452880859</v>
       </c>
       <c r="M7" t="n">
-        <v>-70.43133544921875</v>
+        <v>-54.4282341003418</v>
       </c>
       <c r="N7" t="n">
-        <v>-64.98367309570312</v>
+        <v>-46.24619674682617</v>
       </c>
       <c r="O7" t="n">
-        <v>-73.48676300048828</v>
+        <v>-50.92034149169922</v>
       </c>
       <c r="P7" t="n">
-        <v>-68.98549652099609</v>
+        <v>-48.57260513305664</v>
       </c>
       <c r="Q7" t="n">
-        <v>-70.99674987792969</v>
+        <v>-49.75765228271484</v>
       </c>
       <c r="R7" t="n">
-        <v>-69.40586853027344</v>
+        <v>-51.11204528808594</v>
       </c>
       <c r="S7" t="n">
-        <v>-71.67861938476562</v>
+        <v>-52.55612182617188</v>
       </c>
       <c r="T7" t="n">
-        <v>-74.22937774658203</v>
+        <v>-52.98968505859375</v>
       </c>
       <c r="U7" t="n">
-        <v>-72.90596008300781</v>
+        <v>-54.19139862060547</v>
       </c>
       <c r="V7" t="n">
-        <v>-70.73823547363281</v>
+        <v>-52.23403167724609</v>
       </c>
       <c r="W7" t="n">
-        <v>-71.40110778808594</v>
+        <v>-54.4010124206543</v>
       </c>
       <c r="X7" t="n">
-        <v>-77.80155181884766</v>
+        <v>-49.26727294921875</v>
       </c>
       <c r="Y7" t="n">
-        <v>-76.63549041748047</v>
+        <v>-53.65781784057617</v>
       </c>
       <c r="Z7" t="n">
-        <v>-79.18204498291016</v>
+        <v>-58.41410064697266</v>
       </c>
       <c r="AA7" t="n">
-        <v>-80.08013153076172</v>
+        <v>-55.72740936279297</v>
       </c>
       <c r="AB7" t="n">
-        <v>-83.80258941650391</v>
+        <v>-55.60271453857422</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>-51.17599487304688</v>
+        <v>-44.45858764648438</v>
       </c>
       <c r="B8" t="n">
-        <v>-53.59403610229492</v>
+        <v>-44.25540924072266</v>
       </c>
       <c r="C8" t="n">
-        <v>-58.62064361572266</v>
+        <v>-43.74545288085938</v>
       </c>
       <c r="D8" t="n">
-        <v>-60.28693389892578</v>
+        <v>-45.87172698974609</v>
       </c>
       <c r="E8" t="n">
-        <v>-59.97678756713867</v>
+        <v>-43.96171188354492</v>
       </c>
       <c r="F8" t="n">
-        <v>-54.9075813293457</v>
+        <v>-45.97286605834961</v>
       </c>
       <c r="G8" t="n">
-        <v>-60.8218994140625</v>
+        <v>-47.42250442504883</v>
       </c>
       <c r="H8" t="n">
-        <v>-59.519287109375</v>
+        <v>-45.85314178466797</v>
       </c>
       <c r="I8" t="n">
-        <v>-62.35908889770508</v>
+        <v>-48.96924209594727</v>
       </c>
       <c r="J8" t="n">
-        <v>-64.10920715332031</v>
+        <v>-46.9132080078125</v>
       </c>
       <c r="K8" t="n">
-        <v>-66.239013671875</v>
+        <v>-51.83929443359375</v>
       </c>
       <c r="L8" t="n">
-        <v>-66.88768005371094</v>
+        <v>-48.4498291015625</v>
       </c>
       <c r="M8" t="n">
-        <v>-68.73649597167969</v>
+        <v>-50.18611907958984</v>
       </c>
       <c r="N8" t="n">
-        <v>-65.59660339355469</v>
+        <v>-48.47720718383789</v>
       </c>
       <c r="O8" t="n">
-        <v>-70.37828063964844</v>
+        <v>-53.0195198059082</v>
       </c>
       <c r="P8" t="n">
-        <v>-68.01747131347656</v>
+        <v>-53.72293853759766</v>
       </c>
       <c r="Q8" t="n">
-        <v>-67.61648559570312</v>
+        <v>-52.75686645507812</v>
       </c>
       <c r="R8" t="n">
-        <v>-71.669677734375</v>
+        <v>-52.73811721801758</v>
       </c>
       <c r="S8" t="n">
-        <v>-71.67903137207031</v>
+        <v>-51.50477981567383</v>
       </c>
       <c r="T8" t="n">
-        <v>-73.30935668945312</v>
+        <v>-54.09079742431641</v>
       </c>
       <c r="U8" t="n">
-        <v>-69.37790679931641</v>
+        <v>-52.62389373779297</v>
       </c>
       <c r="V8" t="n">
-        <v>-75.74718475341797</v>
+        <v>-53.69901657104492</v>
       </c>
       <c r="W8" t="n">
-        <v>-71.088623046875</v>
+        <v>-54.2218017578125</v>
       </c>
       <c r="X8" t="n">
-        <v>-72.48165130615234</v>
+        <v>-56.57583618164062</v>
       </c>
       <c r="Y8" t="n">
-        <v>-76.87666320800781</v>
+        <v>-53.90227127075195</v>
       </c>
       <c r="Z8" t="n">
-        <v>-76.08159637451172</v>
+        <v>-51.38205718994141</v>
       </c>
       <c r="AA8" t="n">
-        <v>-77.36408233642578</v>
+        <v>-54.3906135559082</v>
       </c>
       <c r="AB8" t="n">
-        <v>-82.48197937011719</v>
+        <v>-51.83428192138672</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>-59.0591926574707</v>
+        <v>-44.66403198242188</v>
       </c>
       <c r="B9" t="n">
-        <v>-61.37171173095703</v>
+        <v>-45.29808807373047</v>
       </c>
       <c r="C9" t="n">
-        <v>-58.87860107421875</v>
+        <v>-45.10898971557617</v>
       </c>
       <c r="D9" t="n">
-        <v>-60.83354949951172</v>
+        <v>-47.71498107910156</v>
       </c>
       <c r="E9" t="n">
-        <v>-63.73352813720703</v>
+        <v>-45.70597839355469</v>
       </c>
       <c r="F9" t="n">
-        <v>-61.41115570068359</v>
+        <v>-47.09680938720703</v>
       </c>
       <c r="G9" t="n">
-        <v>-61.0620002746582</v>
+        <v>-47.5026969909668</v>
       </c>
       <c r="H9" t="n">
-        <v>-65.3858642578125</v>
+        <v>-48.38098907470703</v>
       </c>
       <c r="I9" t="n">
-        <v>-59.90016555786133</v>
+        <v>-46.61978149414062</v>
       </c>
       <c r="J9" t="n">
-        <v>-63.9287109375</v>
+        <v>-51.20893478393555</v>
       </c>
       <c r="K9" t="n">
-        <v>-66.41543579101562</v>
+        <v>-49.2418327331543</v>
       </c>
       <c r="L9" t="n">
-        <v>-64.75648498535156</v>
+        <v>-47.6416015625</v>
       </c>
       <c r="M9" t="n">
-        <v>-67.22151947021484</v>
+        <v>-52.03745651245117</v>
       </c>
       <c r="N9" t="n">
-        <v>-64.55165100097656</v>
+        <v>-52.97294998168945</v>
       </c>
       <c r="O9" t="n">
-        <v>-72.41883087158203</v>
+        <v>-54.36359405517578</v>
       </c>
       <c r="P9" t="n">
-        <v>-69.34128570556641</v>
+        <v>-52.6606330871582</v>
       </c>
       <c r="Q9" t="n">
-        <v>-68.46666717529297</v>
+        <v>-55.86273193359375</v>
       </c>
       <c r="R9" t="n">
-        <v>-68.18747711181641</v>
+        <v>-53.16482543945312</v>
       </c>
       <c r="S9" t="n">
-        <v>-71.89634704589844</v>
+        <v>-53.9349479675293</v>
       </c>
       <c r="T9" t="n">
-        <v>-72.26173400878906</v>
+        <v>-54.6314697265625</v>
       </c>
       <c r="U9" t="n">
-        <v>-73.2772216796875</v>
+        <v>-51.4801025390625</v>
       </c>
       <c r="V9" t="n">
-        <v>-72.62757873535156</v>
+        <v>-52.78258514404297</v>
       </c>
       <c r="W9" t="n">
-        <v>-75.14509582519531</v>
+        <v>-52.32088088989258</v>
       </c>
       <c r="X9" t="n">
-        <v>-72.71028900146484</v>
+        <v>-53.01553344726562</v>
       </c>
       <c r="Y9" t="n">
-        <v>-70.92545318603516</v>
+        <v>-53.86494827270508</v>
       </c>
       <c r="Z9" t="n">
-        <v>-78.7479248046875</v>
+        <v>-53.30454254150391</v>
       </c>
       <c r="AA9" t="n">
-        <v>-73.73227691650391</v>
+        <v>-55.30101776123047</v>
       </c>
       <c r="AB9" t="n">
-        <v>-80.90633392333984</v>
+        <v>-57.9416389465332</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>-55.5160026550293</v>
+        <v>-39.12181091308594</v>
       </c>
       <c r="B10" t="n">
-        <v>-59.32087326049805</v>
+        <v>-46.64934921264648</v>
       </c>
       <c r="C10" t="n">
-        <v>-55.69062042236328</v>
+        <v>-45.1938591003418</v>
       </c>
       <c r="D10" t="n">
-        <v>-59.43877029418945</v>
+        <v>-48.27265167236328</v>
       </c>
       <c r="E10" t="n">
-        <v>-59.63532257080078</v>
+        <v>-50.68456268310547</v>
       </c>
       <c r="F10" t="n">
-        <v>-60.69965744018555</v>
+        <v>-45.89110946655273</v>
       </c>
       <c r="G10" t="n">
-        <v>-63.22006225585938</v>
+        <v>-46.09725952148438</v>
       </c>
       <c r="H10" t="n">
-        <v>-61.77261352539062</v>
+        <v>-48.12667465209961</v>
       </c>
       <c r="I10" t="n">
-        <v>-65.58724975585938</v>
+        <v>-47.01843643188477</v>
       </c>
       <c r="J10" t="n">
-        <v>-59.88871002197266</v>
+        <v>-50.17618560791016</v>
       </c>
       <c r="K10" t="n">
-        <v>-67.08258819580078</v>
+        <v>-48.57525634765625</v>
       </c>
       <c r="L10" t="n">
-        <v>-69.80506134033203</v>
+        <v>-53.5469856262207</v>
       </c>
       <c r="M10" t="n">
-        <v>-68.08821105957031</v>
+        <v>-50.12737274169922</v>
       </c>
       <c r="N10" t="n">
-        <v>-66.73162841796875</v>
+        <v>-54.78336334228516</v>
       </c>
       <c r="O10" t="n">
-        <v>-67.13804626464844</v>
+        <v>-53.8497314453125</v>
       </c>
       <c r="P10" t="n">
-        <v>-72.51000213623047</v>
+        <v>-52.02029418945312</v>
       </c>
       <c r="Q10" t="n">
-        <v>-72.82742309570312</v>
+        <v>-50.90266799926758</v>
       </c>
       <c r="R10" t="n">
-        <v>-71.77513122558594</v>
+        <v>-50.06453704833984</v>
       </c>
       <c r="S10" t="n">
-        <v>-77.37395477294922</v>
+        <v>-53.68118286132812</v>
       </c>
       <c r="T10" t="n">
-        <v>-75.65969848632812</v>
+        <v>-54.89473724365234</v>
       </c>
       <c r="U10" t="n">
-        <v>-66.03615570068359</v>
+        <v>-56.57947540283203</v>
       </c>
       <c r="V10" t="n">
-        <v>-68.30891418457031</v>
+        <v>-55.93012619018555</v>
       </c>
       <c r="W10" t="n">
-        <v>-79.10562896728516</v>
+        <v>-54.77272796630859</v>
       </c>
       <c r="X10" t="n">
-        <v>-70.11925506591797</v>
+        <v>-54.05218505859375</v>
       </c>
       <c r="Y10" t="n">
-        <v>-77.05744934082031</v>
+        <v>-54.90413284301758</v>
       </c>
       <c r="Z10" t="n">
-        <v>-77.67154693603516</v>
+        <v>-55.8582878112793</v>
       </c>
       <c r="AA10" t="n">
-        <v>-82.02568054199219</v>
+        <v>-58.16130447387695</v>
       </c>
       <c r="AB10" t="n">
-        <v>-74.91375732421875</v>
+        <v>-53.4565315246582</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>-56.92237091064453</v>
+        <v>-47.02125549316406</v>
       </c>
       <c r="B11" t="n">
-        <v>-57.29691696166992</v>
+        <v>-46.58137893676758</v>
       </c>
       <c r="C11" t="n">
-        <v>-58.68312835693359</v>
+        <v>-47.22534942626953</v>
       </c>
       <c r="D11" t="n">
-        <v>-60.45308685302734</v>
+        <v>-46.60981750488281</v>
       </c>
       <c r="E11" t="n">
-        <v>-60.08655548095703</v>
+        <v>-49.63618087768555</v>
       </c>
       <c r="F11" t="n">
-        <v>-62.45539474487305</v>
+        <v>-47.89403533935547</v>
       </c>
       <c r="G11" t="n">
-        <v>-60.26737213134766</v>
+        <v>-49.24105072021484</v>
       </c>
       <c r="H11" t="n">
-        <v>-65.65399169921875</v>
+        <v>-52.19019317626953</v>
       </c>
       <c r="I11" t="n">
-        <v>-63.89289474487305</v>
+        <v>-46.71459197998047</v>
       </c>
       <c r="J11" t="n">
-        <v>-59.71577072143555</v>
+        <v>-50.47639846801758</v>
       </c>
       <c r="K11" t="n">
-        <v>-65.20128631591797</v>
+        <v>-47.24239730834961</v>
       </c>
       <c r="L11" t="n">
-        <v>-63.75847244262695</v>
+        <v>-53.22939300537109</v>
       </c>
       <c r="M11" t="n">
-        <v>-70.11396789550781</v>
+        <v>-50.3544921875</v>
       </c>
       <c r="N11" t="n">
-        <v>-69.86952209472656</v>
+        <v>-48.27704620361328</v>
       </c>
       <c r="O11" t="n">
-        <v>-73.65669250488281</v>
+        <v>-52.2994270324707</v>
       </c>
       <c r="P11" t="n">
-        <v>-68.37461853027344</v>
+        <v>-51.86870574951172</v>
       </c>
       <c r="Q11" t="n">
-        <v>-75.03041839599609</v>
+        <v>-52.95248413085938</v>
       </c>
       <c r="R11" t="n">
-        <v>-74.12325286865234</v>
+        <v>-52.68215179443359</v>
       </c>
       <c r="S11" t="n">
-        <v>-73.54981994628906</v>
+        <v>-54.14744186401367</v>
       </c>
       <c r="T11" t="n">
-        <v>-74.35606384277344</v>
+        <v>-54.42976760864258</v>
       </c>
       <c r="U11" t="n">
-        <v>-77.24849700927734</v>
+        <v>-52.95650482177734</v>
       </c>
       <c r="V11" t="n">
-        <v>-74.12379455566406</v>
+        <v>-55.82483673095703</v>
       </c>
       <c r="W11" t="n">
-        <v>-78.06961059570312</v>
+        <v>-54.35262298583984</v>
       </c>
       <c r="X11" t="n">
-        <v>-76.83967590332031</v>
+        <v>-55.69370269775391</v>
       </c>
       <c r="Y11" t="n">
-        <v>-78.64238739013672</v>
+        <v>-55.3239631652832</v>
       </c>
       <c r="Z11" t="n">
-        <v>-80.68653106689453</v>
+        <v>-56.95648956298828</v>
       </c>
       <c r="AA11" t="n">
-        <v>-79.21458435058594</v>
+        <v>-56.28501510620117</v>
       </c>
       <c r="AB11" t="n">
-        <v>-78.15306091308594</v>
+        <v>-57.09693145751953</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>-58.48909378051758</v>
+        <v>-47.32057952880859</v>
       </c>
       <c r="B12" t="n">
-        <v>-61.9114990234375</v>
+        <v>-48.1151123046875</v>
       </c>
       <c r="C12" t="n">
-        <v>-63.41082763671875</v>
+        <v>-45.90510559082031</v>
       </c>
       <c r="D12" t="n">
-        <v>-64.53886413574219</v>
+        <v>-49.08084869384766</v>
       </c>
       <c r="E12" t="n">
-        <v>-62.73616790771484</v>
+        <v>-49.94729995727539</v>
       </c>
       <c r="F12" t="n">
-        <v>-63.28441619873047</v>
+        <v>-50.68285369873047</v>
       </c>
       <c r="G12" t="n">
-        <v>-66.86582946777344</v>
+        <v>-50.95113372802734</v>
       </c>
       <c r="H12" t="n">
-        <v>-66.29201507568359</v>
+        <v>-52.38076782226562</v>
       </c>
       <c r="I12" t="n">
-        <v>-66.02408599853516</v>
+        <v>-47.47702026367188</v>
       </c>
       <c r="J12" t="n">
-        <v>-67.37745666503906</v>
+        <v>-48.8932991027832</v>
       </c>
       <c r="K12" t="n">
-        <v>-61.57733917236328</v>
+        <v>-48.71118545532227</v>
       </c>
       <c r="L12" t="n">
-        <v>-68.89759063720703</v>
+        <v>-51.22174072265625</v>
       </c>
       <c r="M12" t="n">
-        <v>-69.02716827392578</v>
+        <v>-49.00471878051758</v>
       </c>
       <c r="N12" t="n">
-        <v>-69.49871826171875</v>
+        <v>-52.05788040161133</v>
       </c>
       <c r="O12" t="n">
-        <v>-67.45500183105469</v>
+        <v>-51.26788330078125</v>
       </c>
       <c r="P12" t="n">
-        <v>-69.52811431884766</v>
+        <v>-51.9616813659668</v>
       </c>
       <c r="Q12" t="n">
-        <v>-71.65644836425781</v>
+        <v>-54.03864669799805</v>
       </c>
       <c r="R12" t="n">
-        <v>-74.47679138183594</v>
+        <v>-53.4595947265625</v>
       </c>
       <c r="S12" t="n">
-        <v>-73.16814422607422</v>
+        <v>-55.94376373291016</v>
       </c>
       <c r="T12" t="n">
-        <v>-75.67391967773438</v>
+        <v>-56.25168991088867</v>
       </c>
       <c r="U12" t="n">
-        <v>-73.53524780273438</v>
+        <v>-53.57329559326172</v>
       </c>
       <c r="V12" t="n">
-        <v>-76.57199859619141</v>
+        <v>-56.7467155456543</v>
       </c>
       <c r="W12" t="n">
-        <v>-75.16112518310547</v>
+        <v>-52.3035774230957</v>
       </c>
       <c r="X12" t="n">
-        <v>-79.30699157714844</v>
+        <v>-53.90332794189453</v>
       </c>
       <c r="Y12" t="n">
-        <v>-82.85700225830078</v>
+        <v>-54.30168533325195</v>
       </c>
       <c r="Z12" t="n">
-        <v>-75.32565307617188</v>
+        <v>-54.806884765625</v>
       </c>
       <c r="AA12" t="n">
-        <v>-79.69426727294922</v>
+        <v>-55.5299072265625</v>
       </c>
       <c r="AB12" t="n">
-        <v>-85.23415374755859</v>
+        <v>-57.26963043212891</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>-65.90314483642578</v>
+        <v>-47.22951889038086</v>
       </c>
       <c r="B13" t="n">
-        <v>-62.50186920166016</v>
+        <v>-46.4117546081543</v>
       </c>
       <c r="C13" t="n">
-        <v>-61.190673828125</v>
+        <v>-44.74771499633789</v>
       </c>
       <c r="D13" t="n">
-        <v>-62.36211013793945</v>
+        <v>-48.97022247314453</v>
       </c>
       <c r="E13" t="n">
-        <v>-65.27644348144531</v>
+        <v>-49.82147216796875</v>
       </c>
       <c r="F13" t="n">
-        <v>-64.73695373535156</v>
+        <v>-46.24026107788086</v>
       </c>
       <c r="G13" t="n">
-        <v>-64.28559112548828</v>
+        <v>-48.67017364501953</v>
       </c>
       <c r="H13" t="n">
-        <v>-71.27503967285156</v>
+        <v>-52.14723587036133</v>
       </c>
       <c r="I13" t="n">
-        <v>-67.71778869628906</v>
+        <v>-50.37056350708008</v>
       </c>
       <c r="J13" t="n">
-        <v>-61.37406158447266</v>
+        <v>-52.03292083740234</v>
       </c>
       <c r="K13" t="n">
-        <v>-65.10200500488281</v>
+        <v>-48.5875358581543</v>
       </c>
       <c r="L13" t="n">
-        <v>-65.44467926025391</v>
+        <v>-49.95302581787109</v>
       </c>
       <c r="M13" t="n">
-        <v>-67.18739318847656</v>
+        <v>-50.90197372436523</v>
       </c>
       <c r="N13" t="n">
-        <v>-68.36161041259766</v>
+        <v>-54.14835739135742</v>
       </c>
       <c r="O13" t="n">
-        <v>-72.70252227783203</v>
+        <v>-52.00418090820312</v>
       </c>
       <c r="P13" t="n">
-        <v>-72.49720764160156</v>
+        <v>-47.94605255126953</v>
       </c>
       <c r="Q13" t="n">
-        <v>-73.34010314941406</v>
+        <v>-52.76544952392578</v>
       </c>
       <c r="R13" t="n">
-        <v>-79.05167388916016</v>
+        <v>-49.96628570556641</v>
       </c>
       <c r="S13" t="n">
-        <v>-70.13699340820312</v>
+        <v>-52.44472503662109</v>
       </c>
       <c r="T13" t="n">
-        <v>-77.02048492431641</v>
+        <v>-55.5615119934082</v>
       </c>
       <c r="U13" t="n">
-        <v>-84.16352844238281</v>
+        <v>-56.65592575073242</v>
       </c>
       <c r="V13" t="n">
-        <v>-74.85790252685547</v>
+        <v>-55.6765251159668</v>
       </c>
       <c r="W13" t="n">
-        <v>-77.129150390625</v>
+        <v>-53.3101921081543</v>
       </c>
       <c r="X13" t="n">
-        <v>-82.65171051025391</v>
+        <v>-53.7601203918457</v>
       </c>
       <c r="Y13" t="n">
-        <v>-81.35713195800781</v>
+        <v>-55.26053619384766</v>
       </c>
       <c r="Z13" t="n">
-        <v>-79.83195495605469</v>
+        <v>-58.28661346435547</v>
       </c>
       <c r="AA13" t="n">
-        <v>-82.56890869140625</v>
+        <v>-57.93131637573242</v>
       </c>
       <c r="AB13" t="n">
-        <v>-82.90206146240234</v>
+        <v>-55.39469146728516</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>-63.49418258666992</v>
+        <v>-47.49927520751953</v>
       </c>
       <c r="B14" t="n">
-        <v>-60.4561653137207</v>
+        <v>-45.82749557495117</v>
       </c>
       <c r="C14" t="n">
-        <v>-64.21138763427734</v>
+        <v>-50.25790405273438</v>
       </c>
       <c r="D14" t="n">
-        <v>-64.13167572021484</v>
+        <v>-50.47902297973633</v>
       </c>
       <c r="E14" t="n">
-        <v>-70.83878326416016</v>
+        <v>-49.31134033203125</v>
       </c>
       <c r="F14" t="n">
-        <v>-65.23210144042969</v>
+        <v>-49.67377471923828</v>
       </c>
       <c r="G14" t="n">
-        <v>-65.20094299316406</v>
+        <v>-51.81311798095703</v>
       </c>
       <c r="H14" t="n">
-        <v>-67.5638427734375</v>
+        <v>-51.02509689331055</v>
       </c>
       <c r="I14" t="n">
-        <v>-65.57559967041016</v>
+        <v>-54.84840774536133</v>
       </c>
       <c r="J14" t="n">
-        <v>-66.86076354980469</v>
+        <v>-51.90558624267578</v>
       </c>
       <c r="K14" t="n">
-        <v>-68.82637023925781</v>
+        <v>-49.55432510375977</v>
       </c>
       <c r="L14" t="n">
-        <v>-69.60560607910156</v>
+        <v>-53.67982864379883</v>
       </c>
       <c r="M14" t="n">
-        <v>-70.2008056640625</v>
+        <v>-50.16133880615234</v>
       </c>
       <c r="N14" t="n">
-        <v>-71.16615295410156</v>
+        <v>-49.76430892944336</v>
       </c>
       <c r="O14" t="n">
-        <v>-70.60492706298828</v>
+        <v>-53.96170806884766</v>
       </c>
       <c r="P14" t="n">
-        <v>-74.49031066894531</v>
+        <v>-54.1585807800293</v>
       </c>
       <c r="Q14" t="n">
-        <v>-73.19929504394531</v>
+        <v>-54.64727783203125</v>
       </c>
       <c r="R14" t="n">
-        <v>-77.54786682128906</v>
+        <v>-54.147705078125</v>
       </c>
       <c r="S14" t="n">
-        <v>-71.67961120605469</v>
+        <v>-52.84505462646484</v>
       </c>
       <c r="T14" t="n">
-        <v>-75.67070007324219</v>
+        <v>-51.99172210693359</v>
       </c>
       <c r="U14" t="n">
-        <v>-74.53125</v>
+        <v>-53.20928955078125</v>
       </c>
       <c r="V14" t="n">
-        <v>-70.00687408447266</v>
+        <v>-55.54476165771484</v>
       </c>
       <c r="W14" t="n">
-        <v>-77.55565643310547</v>
+        <v>-50.70330047607422</v>
       </c>
       <c r="X14" t="n">
-        <v>-79.15355682373047</v>
+        <v>-53.22603607177734</v>
       </c>
       <c r="Y14" t="n">
-        <v>-76.74304962158203</v>
+        <v>-56.68585968017578</v>
       </c>
       <c r="Z14" t="n">
-        <v>-79.60240173339844</v>
+        <v>-58.62018585205078</v>
       </c>
       <c r="AA14" t="n">
-        <v>-78.29042053222656</v>
+        <v>-55.93502044677734</v>
       </c>
       <c r="AB14" t="n">
-        <v>-84.55947113037109</v>
+        <v>-55.12460327148438</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>-62.30966949462891</v>
+        <v>-50.28752136230469</v>
       </c>
       <c r="B15" t="n">
-        <v>-65.96763610839844</v>
+        <v>-48.19797515869141</v>
       </c>
       <c r="C15" t="n">
-        <v>-68.57225036621094</v>
+        <v>-50.74509811401367</v>
       </c>
       <c r="D15" t="n">
-        <v>-70.42918395996094</v>
+        <v>-49.95989227294922</v>
       </c>
       <c r="E15" t="n">
-        <v>-66.82102966308594</v>
+        <v>-50.29404449462891</v>
       </c>
       <c r="F15" t="n">
-        <v>-67.17020416259766</v>
+        <v>-51.78090286254883</v>
       </c>
       <c r="G15" t="n">
-        <v>-67.83538055419922</v>
+        <v>-52.7792854309082</v>
       </c>
       <c r="H15" t="n">
-        <v>-69.94715118408203</v>
+        <v>-51.85343551635742</v>
       </c>
       <c r="I15" t="n">
-        <v>-63.53704833984375</v>
+        <v>-46.35147094726562</v>
       </c>
       <c r="J15" t="n">
-        <v>-71.72233581542969</v>
+        <v>-53.22740936279297</v>
       </c>
       <c r="K15" t="n">
-        <v>-67.69179534912109</v>
+        <v>-50.39856719970703</v>
       </c>
       <c r="L15" t="n">
-        <v>-72.63126373291016</v>
+        <v>-53.3067512512207</v>
       </c>
       <c r="M15" t="n">
-        <v>-75.83063507080078</v>
+        <v>-50.5528450012207</v>
       </c>
       <c r="N15" t="n">
-        <v>-73.91346740722656</v>
+        <v>-54.63793182373047</v>
       </c>
       <c r="O15" t="n">
-        <v>-71.29120635986328</v>
+        <v>-51.31819534301758</v>
       </c>
       <c r="P15" t="n">
-        <v>-73.90985107421875</v>
+        <v>-64.55559539794922</v>
       </c>
       <c r="Q15" t="n">
-        <v>-72.51887512207031</v>
+        <v>-68.69786071777344</v>
       </c>
       <c r="R15" t="n">
-        <v>-73.01859283447266</v>
+        <v>-64.40249633789062</v>
       </c>
       <c r="S15" t="n">
-        <v>-73.77928161621094</v>
+        <v>-68.73667907714844</v>
       </c>
       <c r="T15" t="n">
-        <v>-77.18952178955078</v>
+        <v>-64.65493011474609</v>
       </c>
       <c r="U15" t="n">
-        <v>-77.90135192871094</v>
+        <v>-66.87474060058594</v>
       </c>
       <c r="V15" t="n">
-        <v>-81.75455474853516</v>
+        <v>-66.82463073730469</v>
       </c>
       <c r="W15" t="n">
-        <v>-78.28952789306641</v>
+        <v>-71.66188049316406</v>
       </c>
       <c r="X15" t="n">
-        <v>-72.85260772705078</v>
+        <v>-70.35524749755859</v>
       </c>
       <c r="Y15" t="n">
-        <v>-76.62331390380859</v>
+        <v>-69.22618103027344</v>
       </c>
       <c r="Z15" t="n">
-        <v>-79.37429809570312</v>
+        <v>-69.90742492675781</v>
       </c>
       <c r="AA15" t="n">
-        <v>-79.42280578613281</v>
+        <v>-69.34880828857422</v>
       </c>
       <c r="AB15" t="n">
-        <v>-86.00511169433594</v>
+        <v>-71.47173309326172</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>-67.877685546875</v>
+        <v>-47.89324188232422</v>
       </c>
       <c r="B16" t="n">
-        <v>-66.19985198974609</v>
+        <v>-48.77280426025391</v>
       </c>
       <c r="C16" t="n">
-        <v>-67.40251159667969</v>
+        <v>-47.33703994750977</v>
       </c>
       <c r="D16" t="n">
-        <v>-74.11466217041016</v>
+        <v>-48.29613494873047</v>
       </c>
       <c r="E16" t="n">
-        <v>-69.12591552734375</v>
+        <v>-49.33088302612305</v>
       </c>
       <c r="F16" t="n">
-        <v>-69.30365753173828</v>
+        <v>-50.8424186706543</v>
       </c>
       <c r="G16" t="n">
-        <v>-68.29499816894531</v>
+        <v>-51.62396240234375</v>
       </c>
       <c r="H16" t="n">
-        <v>-73.26917266845703</v>
+        <v>-55.71799850463867</v>
       </c>
       <c r="I16" t="n">
-        <v>-73.71580505371094</v>
+        <v>-52.55010223388672</v>
       </c>
       <c r="J16" t="n">
-        <v>-75.24391174316406</v>
+        <v>-51.89943695068359</v>
       </c>
       <c r="K16" t="n">
-        <v>-68.81834411621094</v>
+        <v>-51.68509674072266</v>
       </c>
       <c r="L16" t="n">
-        <v>-73.67750549316406</v>
+        <v>-52.66959381103516</v>
       </c>
       <c r="M16" t="n">
-        <v>-72.39320373535156</v>
+        <v>-56.301025390625</v>
       </c>
       <c r="N16" t="n">
-        <v>-73.14854431152344</v>
+        <v>-55.11457061767578</v>
       </c>
       <c r="O16" t="n">
-        <v>-73.93575286865234</v>
+        <v>-53.9765510559082</v>
       </c>
       <c r="P16" t="n">
-        <v>-74.23655700683594</v>
+        <v>-51.9483642578125</v>
       </c>
       <c r="Q16" t="n">
-        <v>-74.09754943847656</v>
+        <v>-67.92775726318359</v>
       </c>
       <c r="R16" t="n">
-        <v>-76.44931793212891</v>
+        <v>-66.52024841308594</v>
       </c>
       <c r="S16" t="n">
-        <v>-74.11637878417969</v>
+        <v>-69.79842376708984</v>
       </c>
       <c r="T16" t="n">
-        <v>-75.38789367675781</v>
+        <v>-70.58229064941406</v>
       </c>
       <c r="U16" t="n">
-        <v>-72.05419158935547</v>
+        <v>-66.39036560058594</v>
       </c>
       <c r="V16" t="n">
-        <v>-78.44207763671875</v>
+        <v>-70.05596160888672</v>
       </c>
       <c r="W16" t="n">
-        <v>-78.82579040527344</v>
+        <v>-68.60011291503906</v>
       </c>
       <c r="X16" t="n">
-        <v>-83.22924041748047</v>
+        <v>-69.43851470947266</v>
       </c>
       <c r="Y16" t="n">
-        <v>-77.67035675048828</v>
+        <v>-67.20568084716797</v>
       </c>
       <c r="Z16" t="n">
-        <v>-80.05003356933594</v>
+        <v>-67.77571868896484</v>
       </c>
       <c r="AA16" t="n">
-        <v>-80.2943115234375</v>
+        <v>-71.20092010498047</v>
       </c>
       <c r="AB16" t="n">
-        <v>-77.62066650390625</v>
+        <v>-68.03513336181641</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>-66.38054656982422</v>
+        <v>-48.64846038818359</v>
       </c>
       <c r="B17" t="n">
-        <v>-72.57728576660156</v>
+        <v>-46.66537094116211</v>
       </c>
       <c r="C17" t="n">
-        <v>-72.18824768066406</v>
+        <v>-48.49109649658203</v>
       </c>
       <c r="D17" t="n">
-        <v>-61.44972610473633</v>
+        <v>-49.96242904663086</v>
       </c>
       <c r="E17" t="n">
-        <v>-70.53150177001953</v>
+        <v>-51.98567962646484</v>
       </c>
       <c r="F17" t="n">
-        <v>-64.85343933105469</v>
+        <v>-50.91937637329102</v>
       </c>
       <c r="G17" t="n">
-        <v>-71.25227355957031</v>
+        <v>-54.87287521362305</v>
       </c>
       <c r="H17" t="n">
-        <v>-69.70243072509766</v>
+        <v>-49.38460540771484</v>
       </c>
       <c r="I17" t="n">
-        <v>-74.94989013671875</v>
+        <v>-50.48985290527344</v>
       </c>
       <c r="J17" t="n">
-        <v>-74.6292724609375</v>
+        <v>-51.86396408081055</v>
       </c>
       <c r="K17" t="n">
-        <v>-69.29833221435547</v>
+        <v>-52.21939086914062</v>
       </c>
       <c r="L17" t="n">
-        <v>-72.13933563232422</v>
+        <v>-51.35604095458984</v>
       </c>
       <c r="M17" t="n">
-        <v>-70.00481414794922</v>
+        <v>-53.53836822509766</v>
       </c>
       <c r="N17" t="n">
-        <v>-73.87464904785156</v>
+        <v>-50.91620635986328</v>
       </c>
       <c r="O17" t="n">
-        <v>-69.13288879394531</v>
+        <v>-54.85881423950195</v>
       </c>
       <c r="P17" t="n">
-        <v>-74.51416015625</v>
+        <v>-53.30976104736328</v>
       </c>
       <c r="Q17" t="n">
-        <v>-73.34513092041016</v>
+        <v>-57.02696990966797</v>
       </c>
       <c r="R17" t="n">
-        <v>-74.68004608154297</v>
+        <v>-65.77300262451172</v>
       </c>
       <c r="S17" t="n">
-        <v>-75.2607421875</v>
+        <v>-65.89887237548828</v>
       </c>
       <c r="T17" t="n">
-        <v>-79.81011962890625</v>
+        <v>-70.76648712158203</v>
       </c>
       <c r="U17" t="n">
-        <v>-74.71172332763672</v>
+        <v>-67.61903381347656</v>
       </c>
       <c r="V17" t="n">
-        <v>-80.33384704589844</v>
+        <v>-69.65459442138672</v>
       </c>
       <c r="W17" t="n">
-        <v>-77.35687255859375</v>
+        <v>-70.40023803710938</v>
       </c>
       <c r="X17" t="n">
-        <v>-78.65464019775391</v>
+        <v>-67.80451965332031</v>
       </c>
       <c r="Y17" t="n">
-        <v>-76.00363159179688</v>
+        <v>-68.13453674316406</v>
       </c>
       <c r="Z17" t="n">
-        <v>-79.52149963378906</v>
+        <v>-71.50521087646484</v>
       </c>
       <c r="AA17" t="n">
-        <v>-80.35894012451172</v>
+        <v>-70.48492431640625</v>
       </c>
       <c r="AB17" t="n">
-        <v>-79.83903503417969</v>
+        <v>-71.12799072265625</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>-66.69111633300781</v>
+        <v>-50.22522354125977</v>
       </c>
       <c r="B18" t="n">
-        <v>-72.02314758300781</v>
+        <v>-52.39974212646484</v>
       </c>
       <c r="C18" t="n">
-        <v>-71.76013946533203</v>
+        <v>-51.24489593505859</v>
       </c>
       <c r="D18" t="n">
-        <v>-72.25702667236328</v>
+        <v>-50.8704719543457</v>
       </c>
       <c r="E18" t="n">
-        <v>-75.75534057617188</v>
+        <v>-48.74613571166992</v>
       </c>
       <c r="F18" t="n">
-        <v>-72.15212249755859</v>
+        <v>-52.0855598449707</v>
       </c>
       <c r="G18" t="n">
-        <v>-70.07462310791016</v>
+        <v>-52.33549880981445</v>
       </c>
       <c r="H18" t="n">
-        <v>-66.1748046875</v>
+        <v>-51.09739303588867</v>
       </c>
       <c r="I18" t="n">
-        <v>-73.90046691894531</v>
+        <v>-53.92757034301758</v>
       </c>
       <c r="J18" t="n">
-        <v>-69.79678344726562</v>
+        <v>-53.32944488525391</v>
       </c>
       <c r="K18" t="n">
-        <v>-69.36789703369141</v>
+        <v>-54.2873420715332</v>
       </c>
       <c r="L18" t="n">
-        <v>-77.43444061279297</v>
+        <v>-54.10322189331055</v>
       </c>
       <c r="M18" t="n">
-        <v>-70.47522735595703</v>
+        <v>-54.9906005859375</v>
       </c>
       <c r="N18" t="n">
-        <v>-79.07201385498047</v>
+        <v>-52.40690994262695</v>
       </c>
       <c r="O18" t="n">
-        <v>-73.74082183837891</v>
+        <v>-56.05599975585938</v>
       </c>
       <c r="P18" t="n">
-        <v>-74.91039276123047</v>
+        <v>-56.90422439575195</v>
       </c>
       <c r="Q18" t="n">
-        <v>-74.53038024902344</v>
+        <v>-53.20668792724609</v>
       </c>
       <c r="R18" t="n">
-        <v>-72.55752563476562</v>
+        <v>-53.0686149597168</v>
       </c>
       <c r="S18" t="n">
-        <v>-72.59864807128906</v>
+        <v>-69.54255676269531</v>
       </c>
       <c r="T18" t="n">
-        <v>-72.41017150878906</v>
+        <v>-67.00211334228516</v>
       </c>
       <c r="U18" t="n">
-        <v>-77.51871490478516</v>
+        <v>-68.93470001220703</v>
       </c>
       <c r="V18" t="n">
-        <v>-76.79765319824219</v>
+        <v>-72.82270812988281</v>
       </c>
       <c r="W18" t="n">
-        <v>-78.60032653808594</v>
+        <v>-72.58129119873047</v>
       </c>
       <c r="X18" t="n">
-        <v>-70.48684692382812</v>
+        <v>-68.9930419921875</v>
       </c>
       <c r="Y18" t="n">
-        <v>-76.809326171875</v>
+        <v>-74.2125244140625</v>
       </c>
       <c r="Z18" t="n">
-        <v>-80.16561126708984</v>
+        <v>-71.84358215332031</v>
       </c>
       <c r="AA18" t="n">
-        <v>-80.76869201660156</v>
+        <v>-73.88484191894531</v>
       </c>
       <c r="AB18" t="n">
-        <v>-77.27940368652344</v>
+        <v>-69.86763000488281</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>-65.66892242431641</v>
+        <v>-51.8220100402832</v>
       </c>
       <c r="B19" t="n">
-        <v>-75.6976318359375</v>
+        <v>-54.0688591003418</v>
       </c>
       <c r="C19" t="n">
-        <v>-71.51641082763672</v>
+        <v>-53.62754440307617</v>
       </c>
       <c r="D19" t="n">
-        <v>-68.6466064453125</v>
+        <v>-51.00857543945312</v>
       </c>
       <c r="E19" t="n">
-        <v>-73.03321075439453</v>
+        <v>-52.21724319458008</v>
       </c>
       <c r="F19" t="n">
-        <v>-66.02442932128906</v>
+        <v>-51.45005416870117</v>
       </c>
       <c r="G19" t="n">
-        <v>-71.10191345214844</v>
+        <v>-53.64345550537109</v>
       </c>
       <c r="H19" t="n">
-        <v>-69.96049499511719</v>
+        <v>-51.31417846679688</v>
       </c>
       <c r="I19" t="n">
-        <v>-71.16014862060547</v>
+        <v>-54.69671630859375</v>
       </c>
       <c r="J19" t="n">
-        <v>-73.12614440917969</v>
+        <v>-55.79241943359375</v>
       </c>
       <c r="K19" t="n">
-        <v>-71.51950073242188</v>
+        <v>-49.70817947387695</v>
       </c>
       <c r="L19" t="n">
-        <v>-77.70277404785156</v>
+        <v>-53.22660446166992</v>
       </c>
       <c r="M19" t="n">
-        <v>-72.07955932617188</v>
+        <v>-54.73433303833008</v>
       </c>
       <c r="N19" t="n">
-        <v>-76.76769256591797</v>
+        <v>-53.19573974609375</v>
       </c>
       <c r="O19" t="n">
-        <v>-75.69742584228516</v>
+        <v>-53.80254364013672</v>
       </c>
       <c r="P19" t="n">
-        <v>-78.07212829589844</v>
+        <v>-56.6111946105957</v>
       </c>
       <c r="Q19" t="n">
-        <v>-74.37855529785156</v>
+        <v>-53.1603889465332</v>
       </c>
       <c r="R19" t="n">
-        <v>-74.05214691162109</v>
+        <v>-54.00318145751953</v>
       </c>
       <c r="S19" t="n">
-        <v>-77.59681701660156</v>
+        <v>-52.40974044799805</v>
       </c>
       <c r="T19" t="n">
-        <v>-79.11094665527344</v>
+        <v>-67.6348876953125</v>
       </c>
       <c r="U19" t="n">
-        <v>-79.68849945068359</v>
+        <v>-69.45948791503906</v>
       </c>
       <c r="V19" t="n">
-        <v>-78.59841918945312</v>
+        <v>-71.43819427490234</v>
       </c>
       <c r="W19" t="n">
-        <v>-79.71012878417969</v>
+        <v>-70.95841979980469</v>
       </c>
       <c r="X19" t="n">
-        <v>-82.61798858642578</v>
+        <v>-68.02742767333984</v>
       </c>
       <c r="Y19" t="n">
-        <v>-79.61064910888672</v>
+        <v>-70.29704284667969</v>
       </c>
       <c r="Z19" t="n">
-        <v>-81.41543579101562</v>
+        <v>-70.28620910644531</v>
       </c>
       <c r="AA19" t="n">
-        <v>-81.00087738037109</v>
+        <v>-75.09870910644531</v>
       </c>
       <c r="AB19" t="n">
-        <v>-78.55274963378906</v>
+        <v>-72.26210784912109</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>-70.51654815673828</v>
+        <v>-51.86007690429688</v>
       </c>
       <c r="B20" t="n">
-        <v>-70.49613189697266</v>
+        <v>-50.71985244750977</v>
       </c>
       <c r="C20" t="n">
-        <v>-71.48475646972656</v>
+        <v>-52.65346145629883</v>
       </c>
       <c r="D20" t="n">
-        <v>-74.35157012939453</v>
+        <v>-51.3021125793457</v>
       </c>
       <c r="E20" t="n">
-        <v>-72.06267547607422</v>
+        <v>-52.71793746948242</v>
       </c>
       <c r="F20" t="n">
-        <v>-68.75949096679688</v>
+        <v>-51.7596435546875</v>
       </c>
       <c r="G20" t="n">
-        <v>-71.75226593017578</v>
+        <v>-54.6197395324707</v>
       </c>
       <c r="H20" t="n">
-        <v>-75.00750732421875</v>
+        <v>-52.5129280090332</v>
       </c>
       <c r="I20" t="n">
-        <v>-74.40789794921875</v>
+        <v>-49.82367324829102</v>
       </c>
       <c r="J20" t="n">
-        <v>-69.00860595703125</v>
+        <v>-52.21096038818359</v>
       </c>
       <c r="K20" t="n">
-        <v>-71.31169891357422</v>
+        <v>-52.77191162109375</v>
       </c>
       <c r="L20" t="n">
-        <v>-73.45387268066406</v>
+        <v>-55.56705856323242</v>
       </c>
       <c r="M20" t="n">
-        <v>-79.33461761474609</v>
+        <v>-51.00131988525391</v>
       </c>
       <c r="N20" t="n">
-        <v>-74.49898529052734</v>
+        <v>-57.55972290039062</v>
       </c>
       <c r="O20" t="n">
-        <v>-77.26109313964844</v>
+        <v>-55.5323600769043</v>
       </c>
       <c r="P20" t="n">
-        <v>-73.34968566894531</v>
+        <v>-54.222412109375</v>
       </c>
       <c r="Q20" t="n">
-        <v>-76.31936645507812</v>
+        <v>-56.64765167236328</v>
       </c>
       <c r="R20" t="n">
-        <v>-79.68821716308594</v>
+        <v>-56.49523162841797</v>
       </c>
       <c r="S20" t="n">
-        <v>-77.81813812255859</v>
+        <v>-55.24657440185547</v>
       </c>
       <c r="T20" t="n">
-        <v>-75.16345977783203</v>
+        <v>-56.3955192565918</v>
       </c>
       <c r="U20" t="n">
-        <v>-79.75334167480469</v>
+        <v>-72.59904479980469</v>
       </c>
       <c r="V20" t="n">
-        <v>-77.74275207519531</v>
+        <v>-68.02433776855469</v>
       </c>
       <c r="W20" t="n">
-        <v>-76.28648376464844</v>
+        <v>-68.01971435546875</v>
       </c>
       <c r="X20" t="n">
-        <v>-75.89604187011719</v>
+        <v>-71.76333618164062</v>
       </c>
       <c r="Y20" t="n">
-        <v>-81.85404968261719</v>
+        <v>-72.33756256103516</v>
       </c>
       <c r="Z20" t="n">
-        <v>-78.55402374267578</v>
+        <v>-71.67333984375</v>
       </c>
       <c r="AA20" t="n">
-        <v>-79.07398986816406</v>
+        <v>-69.76461029052734</v>
       </c>
       <c r="AB20" t="n">
-        <v>-83.650634765625</v>
+        <v>-70.05943298339844</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>-71.63816833496094</v>
+        <v>-52.76316452026367</v>
       </c>
       <c r="B21" t="n">
-        <v>-69.71632385253906</v>
+        <v>-52.73208618164062</v>
       </c>
       <c r="C21" t="n">
-        <v>-69.17899322509766</v>
+        <v>-49.40773773193359</v>
       </c>
       <c r="D21" t="n">
-        <v>-77.51766204833984</v>
+        <v>-52.82772064208984</v>
       </c>
       <c r="E21" t="n">
-        <v>-73.50392150878906</v>
+        <v>-52.23093795776367</v>
       </c>
       <c r="F21" t="n">
-        <v>-73.14151000976562</v>
+        <v>-49.32870483398438</v>
       </c>
       <c r="G21" t="n">
-        <v>-67.53705596923828</v>
+        <v>-53.15692901611328</v>
       </c>
       <c r="H21" t="n">
-        <v>-72.12450408935547</v>
+        <v>-52.86566925048828</v>
       </c>
       <c r="I21" t="n">
-        <v>-77.87306213378906</v>
+        <v>-51.0093994140625</v>
       </c>
       <c r="J21" t="n">
-        <v>-71.49028778076172</v>
+        <v>-55.31232833862305</v>
       </c>
       <c r="K21" t="n">
-        <v>-76.09183502197266</v>
+        <v>-52.95493316650391</v>
       </c>
       <c r="L21" t="n">
-        <v>-79.84092712402344</v>
+        <v>-52.73116302490234</v>
       </c>
       <c r="M21" t="n">
-        <v>-73.81364440917969</v>
+        <v>-53.58528900146484</v>
       </c>
       <c r="N21" t="n">
-        <v>-75.14064025878906</v>
+        <v>-52.65914154052734</v>
       </c>
       <c r="O21" t="n">
-        <v>-79.36132049560547</v>
+        <v>-51.91030120849609</v>
       </c>
       <c r="P21" t="n">
-        <v>-74.70512390136719</v>
+        <v>-57.43411254882812</v>
       </c>
       <c r="Q21" t="n">
-        <v>-71.05899047851562</v>
+        <v>-52.95670318603516</v>
       </c>
       <c r="R21" t="n">
-        <v>-75.71920776367188</v>
+        <v>-55.65864181518555</v>
       </c>
       <c r="S21" t="n">
-        <v>-77.61579895019531</v>
+        <v>-54.75880813598633</v>
       </c>
       <c r="T21" t="n">
-        <v>-76.25758361816406</v>
+        <v>-56.77223968505859</v>
       </c>
       <c r="U21" t="n">
-        <v>-79.8961181640625</v>
+        <v>-55.72560882568359</v>
       </c>
       <c r="V21" t="n">
-        <v>-77.63011169433594</v>
+        <v>-70.88741302490234</v>
       </c>
       <c r="W21" t="n">
-        <v>-77.94265747070312</v>
+        <v>-68.90652465820312</v>
       </c>
       <c r="X21" t="n">
-        <v>-80.70580291748047</v>
+        <v>-69.91450500488281</v>
       </c>
       <c r="Y21" t="n">
-        <v>-79.0872802734375</v>
+        <v>-72.42574310302734</v>
       </c>
       <c r="Z21" t="n">
-        <v>-78.93019866943359</v>
+        <v>-69.37944030761719</v>
       </c>
       <c r="AA21" t="n">
-        <v>-80.25437927246094</v>
+        <v>-70.20404052734375</v>
       </c>
       <c r="AB21" t="n">
-        <v>-84.97608184814453</v>
+        <v>-67.81252288818359</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>-73.16664123535156</v>
+        <v>-51.86664962768555</v>
       </c>
       <c r="B22" t="n">
-        <v>-76.08524322509766</v>
+        <v>-52.3482666015625</v>
       </c>
       <c r="C22" t="n">
-        <v>-74.96018981933594</v>
+        <v>-51.4198112487793</v>
       </c>
       <c r="D22" t="n">
-        <v>-72.6575927734375</v>
+        <v>-50.91972351074219</v>
       </c>
       <c r="E22" t="n">
-        <v>-73.88963317871094</v>
+        <v>-50.85391616821289</v>
       </c>
       <c r="F22" t="n">
-        <v>-72.26884460449219</v>
+        <v>-54.93390655517578</v>
       </c>
       <c r="G22" t="n">
-        <v>-73.46075439453125</v>
+        <v>-51.68154144287109</v>
       </c>
       <c r="H22" t="n">
-        <v>-78.10478210449219</v>
+        <v>-48.83151626586914</v>
       </c>
       <c r="I22" t="n">
-        <v>-73.57621765136719</v>
+        <v>-55.34709548950195</v>
       </c>
       <c r="J22" t="n">
-        <v>-74.68040466308594</v>
+        <v>-54.06611251831055</v>
       </c>
       <c r="K22" t="n">
-        <v>-70.11716461181641</v>
+        <v>-53.40439605712891</v>
       </c>
       <c r="L22" t="n">
-        <v>-75.81221771240234</v>
+        <v>-54.25374221801758</v>
       </c>
       <c r="M22" t="n">
-        <v>-76.89328002929688</v>
+        <v>-53.3216667175293</v>
       </c>
       <c r="N22" t="n">
-        <v>-74.36268615722656</v>
+        <v>-54.32076263427734</v>
       </c>
       <c r="O22" t="n">
-        <v>-83.58219909667969</v>
+        <v>-57.45117950439453</v>
       </c>
       <c r="P22" t="n">
-        <v>-77.94508361816406</v>
+        <v>-55.34222412109375</v>
       </c>
       <c r="Q22" t="n">
-        <v>-70.45671081542969</v>
+        <v>-57.0357666015625</v>
       </c>
       <c r="R22" t="n">
-        <v>-73.67375946044922</v>
+        <v>-54.44559478759766</v>
       </c>
       <c r="S22" t="n">
-        <v>-80.00267028808594</v>
+        <v>-56.39290618896484</v>
       </c>
       <c r="T22" t="n">
-        <v>-77.2354736328125</v>
+        <v>-55.75325775146484</v>
       </c>
       <c r="U22" t="n">
-        <v>-69.99967193603516</v>
+        <v>-57.2446403503418</v>
       </c>
       <c r="V22" t="n">
-        <v>-76.76461029052734</v>
+        <v>-57.35049438476562</v>
       </c>
       <c r="W22" t="n">
-        <v>-79.16471862792969</v>
+        <v>-72.70272064208984</v>
       </c>
       <c r="X22" t="n">
-        <v>-79.52717590332031</v>
+        <v>-72.92958068847656</v>
       </c>
       <c r="Y22" t="n">
-        <v>-79.43270874023438</v>
+        <v>-69.69307708740234</v>
       </c>
       <c r="Z22" t="n">
-        <v>-79.33701324462891</v>
+        <v>-69.01883697509766</v>
       </c>
       <c r="AA22" t="n">
-        <v>-73.364013671875</v>
+        <v>-68.63764953613281</v>
       </c>
       <c r="AB22" t="n">
-        <v>-81.99134063720703</v>
+        <v>-73.05783843994141</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>-75.80809783935547</v>
+        <v>-54.61175537109375</v>
       </c>
       <c r="B23" t="n">
-        <v>-76.65592956542969</v>
+        <v>-51.81267166137695</v>
       </c>
       <c r="C23" t="n">
-        <v>-80.40056610107422</v>
+        <v>-52.98918533325195</v>
       </c>
       <c r="D23" t="n">
-        <v>-77.46632385253906</v>
+        <v>-55.14949798583984</v>
       </c>
       <c r="E23" t="n">
-        <v>-71.95722961425781</v>
+        <v>-53.17409133911133</v>
       </c>
       <c r="F23" t="n">
-        <v>-74.95726776123047</v>
+        <v>-53.35282135009766</v>
       </c>
       <c r="G23" t="n">
-        <v>-74.93435668945312</v>
+        <v>-51.93437576293945</v>
       </c>
       <c r="H23" t="n">
-        <v>-75.90707397460938</v>
+        <v>-55.8218879699707</v>
       </c>
       <c r="I23" t="n">
-        <v>-78.75736236572266</v>
+        <v>-56.22738647460938</v>
       </c>
       <c r="J23" t="n">
-        <v>-76.49394989013672</v>
+        <v>-56.48784255981445</v>
       </c>
       <c r="K23" t="n">
-        <v>-70.66416168212891</v>
+        <v>-55.13801956176758</v>
       </c>
       <c r="L23" t="n">
-        <v>-76.57572174072266</v>
+        <v>-55.8057746887207</v>
       </c>
       <c r="M23" t="n">
-        <v>-76.74633026123047</v>
+        <v>-55.57235717773438</v>
       </c>
       <c r="N23" t="n">
-        <v>-73.70371246337891</v>
+        <v>-59.55754852294922</v>
       </c>
       <c r="O23" t="n">
-        <v>-73.87977600097656</v>
+        <v>-57.44136810302734</v>
       </c>
       <c r="P23" t="n">
-        <v>-74.77850341796875</v>
+        <v>-57.64064407348633</v>
       </c>
       <c r="Q23" t="n">
-        <v>-76.74845886230469</v>
+        <v>-55.66021728515625</v>
       </c>
       <c r="R23" t="n">
-        <v>-79.56447601318359</v>
+        <v>-57.94157791137695</v>
       </c>
       <c r="S23" t="n">
-        <v>-82.03951263427734</v>
+        <v>-55.06809234619141</v>
       </c>
       <c r="T23" t="n">
-        <v>-83.19242095947266</v>
+        <v>-57.89089965820312</v>
       </c>
       <c r="U23" t="n">
-        <v>-80.4356689453125</v>
+        <v>-57.5999641418457</v>
       </c>
       <c r="V23" t="n">
-        <v>-81.15925598144531</v>
+        <v>-55.96894073486328</v>
       </c>
       <c r="W23" t="n">
-        <v>-74.35964965820312</v>
+        <v>-54.72615814208984</v>
       </c>
       <c r="X23" t="n">
-        <v>-72.58455657958984</v>
+        <v>-70.33320617675781</v>
       </c>
       <c r="Y23" t="n">
-        <v>-77.21080017089844</v>
+        <v>-68.95033264160156</v>
       </c>
       <c r="Z23" t="n">
-        <v>-80.00856018066406</v>
+        <v>-69.90549468994141</v>
       </c>
       <c r="AA23" t="n">
-        <v>-79.32548522949219</v>
+        <v>-70.53894805908203</v>
       </c>
       <c r="AB23" t="n">
-        <v>-75.54943084716797</v>
+        <v>-69.39640808105469</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>-74.07028198242188</v>
+        <v>-52.19430541992188</v>
       </c>
       <c r="B24" t="n">
-        <v>-75.88597106933594</v>
+        <v>-51.96906661987305</v>
       </c>
       <c r="C24" t="n">
-        <v>-81.87270355224609</v>
+        <v>-53.11777877807617</v>
       </c>
       <c r="D24" t="n">
-        <v>-75.53866577148438</v>
+        <v>-54.74143218994141</v>
       </c>
       <c r="E24" t="n">
-        <v>-76.55022430419922</v>
+        <v>-53.1979866027832</v>
       </c>
       <c r="F24" t="n">
-        <v>-73.89364624023438</v>
+        <v>-52.34109497070312</v>
       </c>
       <c r="G24" t="n">
-        <v>-73.91054534912109</v>
+        <v>-53.9310302734375</v>
       </c>
       <c r="H24" t="n">
-        <v>-75.98516082763672</v>
+        <v>-54.16803741455078</v>
       </c>
       <c r="I24" t="n">
-        <v>-73.47712707519531</v>
+        <v>-51.66147613525391</v>
       </c>
       <c r="J24" t="n">
-        <v>-72.49539947509766</v>
+        <v>-55.41135787963867</v>
       </c>
       <c r="K24" t="n">
-        <v>-74.52955627441406</v>
+        <v>-55.0040283203125</v>
       </c>
       <c r="L24" t="n">
-        <v>-76.05091094970703</v>
+        <v>-56.24602127075195</v>
       </c>
       <c r="M24" t="n">
-        <v>-79.46646881103516</v>
+        <v>-53.08217620849609</v>
       </c>
       <c r="N24" t="n">
-        <v>-76.15562438964844</v>
+        <v>-56.71810913085938</v>
       </c>
       <c r="O24" t="n">
-        <v>-77.7506103515625</v>
+        <v>-56.64687347412109</v>
       </c>
       <c r="P24" t="n">
-        <v>-76.57834625244141</v>
+        <v>-55.54531860351562</v>
       </c>
       <c r="Q24" t="n">
-        <v>-80.03543853759766</v>
+        <v>-55.42816925048828</v>
       </c>
       <c r="R24" t="n">
-        <v>-72.43936157226562</v>
+        <v>-55.80179595947266</v>
       </c>
       <c r="S24" t="n">
-        <v>-80.81486511230469</v>
+        <v>-57.04141235351562</v>
       </c>
       <c r="T24" t="n">
-        <v>-80.46818542480469</v>
+        <v>-57.05416870117188</v>
       </c>
       <c r="U24" t="n">
-        <v>-72.40145111083984</v>
+        <v>-54.4736213684082</v>
       </c>
       <c r="V24" t="n">
-        <v>-81.62532043457031</v>
+        <v>-56.85734176635742</v>
       </c>
       <c r="W24" t="n">
-        <v>-82.2410888671875</v>
+        <v>-55.1370735168457</v>
       </c>
       <c r="X24" t="n">
-        <v>-74.94746398925781</v>
+        <v>-57.75749588012695</v>
       </c>
       <c r="Y24" t="n">
-        <v>-81.07450103759766</v>
+        <v>-69.50279998779297</v>
       </c>
       <c r="Z24" t="n">
-        <v>-76.77145385742188</v>
+        <v>-75.34295654296875</v>
       </c>
       <c r="AA24" t="n">
-        <v>-79.66426849365234</v>
+        <v>-73.65448760986328</v>
       </c>
       <c r="AB24" t="n">
-        <v>-78.9097900390625</v>
+        <v>-70.92965698242188</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>-76.6339111328125</v>
+        <v>-48.77504730224609</v>
       </c>
       <c r="B25" t="n">
-        <v>-76.89310455322266</v>
+        <v>-53.398681640625</v>
       </c>
       <c r="C25" t="n">
-        <v>-73.57195281982422</v>
+        <v>-54.9883918762207</v>
       </c>
       <c r="D25" t="n">
-        <v>-78.45179748535156</v>
+        <v>-55.47389984130859</v>
       </c>
       <c r="E25" t="n">
-        <v>-74.48390197753906</v>
+        <v>-50.65058135986328</v>
       </c>
       <c r="F25" t="n">
-        <v>-72.8756103515625</v>
+        <v>-50.44338226318359</v>
       </c>
       <c r="G25" t="n">
-        <v>-76.81378173828125</v>
+        <v>-53.81319046020508</v>
       </c>
       <c r="H25" t="n">
-        <v>-71.61107635498047</v>
+        <v>-57.38076019287109</v>
       </c>
       <c r="I25" t="n">
-        <v>-75.9609375</v>
+        <v>-53.24556350708008</v>
       </c>
       <c r="J25" t="n">
-        <v>-69.08363342285156</v>
+        <v>-53.29892730712891</v>
       </c>
       <c r="K25" t="n">
-        <v>-78.69931030273438</v>
+        <v>-56.98215866088867</v>
       </c>
       <c r="L25" t="n">
-        <v>-79.52665710449219</v>
+        <v>-55.66206741333008</v>
       </c>
       <c r="M25" t="n">
-        <v>-76.26544952392578</v>
+        <v>-54.9296875</v>
       </c>
       <c r="N25" t="n">
-        <v>-76.05919647216797</v>
+        <v>-56.30830764770508</v>
       </c>
       <c r="O25" t="n">
-        <v>-81.21054840087891</v>
+        <v>-57.09574127197266</v>
       </c>
       <c r="P25" t="n">
-        <v>-79.39593505859375</v>
+        <v>-54.82368850708008</v>
       </c>
       <c r="Q25" t="n">
-        <v>-82.25514221191406</v>
+        <v>-58.25018310546875</v>
       </c>
       <c r="R25" t="n">
-        <v>-72.0318603515625</v>
+        <v>-55.84614181518555</v>
       </c>
       <c r="S25" t="n">
-        <v>-81.05567932128906</v>
+        <v>-56.07160186767578</v>
       </c>
       <c r="T25" t="n">
-        <v>-81.41032409667969</v>
+        <v>-50.93399429321289</v>
       </c>
       <c r="U25" t="n">
-        <v>-77.55890655517578</v>
+        <v>-57.90365600585938</v>
       </c>
       <c r="V25" t="n">
-        <v>-79.62325286865234</v>
+        <v>-60.25502395629883</v>
       </c>
       <c r="W25" t="n">
-        <v>-79.58866119384766</v>
+        <v>-60.11211395263672</v>
       </c>
       <c r="X25" t="n">
-        <v>-77.59519195556641</v>
+        <v>-56.45001220703125</v>
       </c>
       <c r="Y25" t="n">
-        <v>-81.99845123291016</v>
+        <v>-58.03369140625</v>
       </c>
       <c r="Z25" t="n">
-        <v>-76.82286834716797</v>
+        <v>-70.56272888183594</v>
       </c>
       <c r="AA25" t="n">
-        <v>-79.83009338378906</v>
+        <v>-74.73351287841797</v>
       </c>
       <c r="AB25" t="n">
-        <v>-84.60743713378906</v>
+        <v>-72.53140258789062</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>-79.56044006347656</v>
+        <v>-52.14778900146484</v>
       </c>
       <c r="B26" t="n">
-        <v>-78.52989959716797</v>
+        <v>-50.83913421630859</v>
       </c>
       <c r="C26" t="n">
-        <v>-76.45951843261719</v>
+        <v>-54.84902191162109</v>
       </c>
       <c r="D26" t="n">
-        <v>-76.89188385009766</v>
+        <v>-56.95793533325195</v>
       </c>
       <c r="E26" t="n">
-        <v>-79.49822235107422</v>
+        <v>-51.96546173095703</v>
       </c>
       <c r="F26" t="n">
-        <v>-74.42856597900391</v>
+        <v>-53.24138641357422</v>
       </c>
       <c r="G26" t="n">
-        <v>-79.55971527099609</v>
+        <v>-54.2042121887207</v>
       </c>
       <c r="H26" t="n">
-        <v>-81.63719940185547</v>
+        <v>-55.77830123901367</v>
       </c>
       <c r="I26" t="n">
-        <v>-76.69266510009766</v>
+        <v>-55.86244583129883</v>
       </c>
       <c r="J26" t="n">
-        <v>-79.14131927490234</v>
+        <v>-54.20487213134766</v>
       </c>
       <c r="K26" t="n">
-        <v>-81.19374847412109</v>
+        <v>-55.08611297607422</v>
       </c>
       <c r="L26" t="n">
-        <v>-77.92402648925781</v>
+        <v>-58.04201126098633</v>
       </c>
       <c r="M26" t="n">
-        <v>-79.77883911132812</v>
+        <v>-56.90396118164062</v>
       </c>
       <c r="N26" t="n">
-        <v>-79.90240478515625</v>
+        <v>-53.19670486450195</v>
       </c>
       <c r="O26" t="n">
-        <v>-74.62898254394531</v>
+        <v>-57.4512939453125</v>
       </c>
       <c r="P26" t="n">
-        <v>-79.30819702148438</v>
+        <v>-57.9738883972168</v>
       </c>
       <c r="Q26" t="n">
-        <v>-82.02508544921875</v>
+        <v>-58.69335174560547</v>
       </c>
       <c r="R26" t="n">
-        <v>-82.02677917480469</v>
+        <v>-54.32785797119141</v>
       </c>
       <c r="S26" t="n">
-        <v>-75.99477386474609</v>
+        <v>-55.04790115356445</v>
       </c>
       <c r="T26" t="n">
-        <v>-78.98751068115234</v>
+        <v>-54.99552154541016</v>
       </c>
       <c r="U26" t="n">
-        <v>-73.92124938964844</v>
+        <v>-52.24306488037109</v>
       </c>
       <c r="V26" t="n">
-        <v>-78.29605865478516</v>
+        <v>-54.45438766479492</v>
       </c>
       <c r="W26" t="n">
-        <v>-78.02203369140625</v>
+        <v>-58.28511428833008</v>
       </c>
       <c r="X26" t="n">
-        <v>-78.61019134521484</v>
+        <v>-55.89629364013672</v>
       </c>
       <c r="Y26" t="n">
-        <v>-81.18259429931641</v>
+        <v>-56.69658660888672</v>
       </c>
       <c r="Z26" t="n">
-        <v>-78.49226379394531</v>
+        <v>-58.54105377197266</v>
       </c>
       <c r="AA26" t="n">
-        <v>-79.79507446289062</v>
+        <v>-74.29019927978516</v>
       </c>
       <c r="AB26" t="n">
-        <v>-81.22373962402344</v>
+        <v>-70.38643646240234</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>-73.36844635009766</v>
+        <v>-57.5158576965332</v>
       </c>
       <c r="B27" t="n">
-        <v>-77.19682312011719</v>
+        <v>-55.49120330810547</v>
       </c>
       <c r="C27" t="n">
-        <v>-78.82787322998047</v>
+        <v>-53.33394622802734</v>
       </c>
       <c r="D27" t="n">
-        <v>-79.00032043457031</v>
+        <v>-52.5635871887207</v>
       </c>
       <c r="E27" t="n">
-        <v>-76.50749969482422</v>
+        <v>-56.56888961791992</v>
       </c>
       <c r="F27" t="n">
-        <v>-82.56536865234375</v>
+        <v>-54.5594596862793</v>
       </c>
       <c r="G27" t="n">
-        <v>-78.51487731933594</v>
+        <v>-56.66851806640625</v>
       </c>
       <c r="H27" t="n">
-        <v>-78.30803680419922</v>
+        <v>-56.2935791015625</v>
       </c>
       <c r="I27" t="n">
-        <v>-76.65489196777344</v>
+        <v>-56.19706344604492</v>
       </c>
       <c r="J27" t="n">
-        <v>-75.03974914550781</v>
+        <v>-57.14913940429688</v>
       </c>
       <c r="K27" t="n">
-        <v>-74.1781005859375</v>
+        <v>-56.83437347412109</v>
       </c>
       <c r="L27" t="n">
-        <v>-79.88047027587891</v>
+        <v>-53.30596923828125</v>
       </c>
       <c r="M27" t="n">
-        <v>-74.26854705810547</v>
+        <v>-53.83443450927734</v>
       </c>
       <c r="N27" t="n">
-        <v>-75.88855743408203</v>
+        <v>-55.21277618408203</v>
       </c>
       <c r="O27" t="n">
-        <v>-84.16246032714844</v>
+        <v>-56.5864372253418</v>
       </c>
       <c r="P27" t="n">
-        <v>-83.58545684814453</v>
+        <v>-56.5009765625</v>
       </c>
       <c r="Q27" t="n">
-        <v>-79.28048706054688</v>
+        <v>-57.05280303955078</v>
       </c>
       <c r="R27" t="n">
-        <v>-78.08992767333984</v>
+        <v>-56.52701568603516</v>
       </c>
       <c r="S27" t="n">
-        <v>-80.3148193359375</v>
+        <v>-60.17999267578125</v>
       </c>
       <c r="T27" t="n">
-        <v>-82.04225158691406</v>
+        <v>-55.94407272338867</v>
       </c>
       <c r="U27" t="n">
-        <v>-77.35020446777344</v>
+        <v>-56.00505828857422</v>
       </c>
       <c r="V27" t="n">
-        <v>-77.93212890625</v>
+        <v>-56.87162017822266</v>
       </c>
       <c r="W27" t="n">
-        <v>-82.75068664550781</v>
+        <v>-57.93756103515625</v>
       </c>
       <c r="X27" t="n">
-        <v>-80.12519836425781</v>
+        <v>-56.69522857666016</v>
       </c>
       <c r="Y27" t="n">
-        <v>-79.90282440185547</v>
+        <v>-58.19617462158203</v>
       </c>
       <c r="Z27" t="n">
-        <v>-80.65210723876953</v>
+        <v>-58.39019775390625</v>
       </c>
       <c r="AA27" t="n">
-        <v>-82.09708404541016</v>
+        <v>-57.28415679931641</v>
       </c>
       <c r="AB27" t="n">
-        <v>-82.69106292724609</v>
+        <v>-70.70953369140625</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>-77.12129211425781</v>
+        <v>-57.16726684570312</v>
       </c>
       <c r="B28" t="n">
-        <v>-81.33280944824219</v>
+        <v>-54.3053092956543</v>
       </c>
       <c r="C28" t="n">
-        <v>-77.17927551269531</v>
+        <v>-55.60681915283203</v>
       </c>
       <c r="D28" t="n">
-        <v>-76.99478912353516</v>
+        <v>-55.0156135559082</v>
       </c>
       <c r="E28" t="n">
-        <v>-79.74996948242188</v>
+        <v>-55.93761444091797</v>
       </c>
       <c r="F28" t="n">
-        <v>-77.31790924072266</v>
+        <v>-57.15389251708984</v>
       </c>
       <c r="G28" t="n">
-        <v>-77.37118530273438</v>
+        <v>-53.85092926025391</v>
       </c>
       <c r="H28" t="n">
-        <v>-76.58278656005859</v>
+        <v>-57.5140380859375</v>
       </c>
       <c r="I28" t="n">
-        <v>-81.98173522949219</v>
+        <v>-55.10968017578125</v>
       </c>
       <c r="J28" t="n">
-        <v>-78.80445098876953</v>
+        <v>-56.17216873168945</v>
       </c>
       <c r="K28" t="n">
-        <v>-76.84877014160156</v>
+        <v>-51.51703643798828</v>
       </c>
       <c r="L28" t="n">
-        <v>-75.07277679443359</v>
+        <v>-53.84310150146484</v>
       </c>
       <c r="M28" t="n">
-        <v>-79.77114868164062</v>
+        <v>-57.86371994018555</v>
       </c>
       <c r="N28" t="n">
-        <v>-78.32823181152344</v>
+        <v>-56.8032341003418</v>
       </c>
       <c r="O28" t="n">
-        <v>-82.10035705566406</v>
+        <v>-55.06230545043945</v>
       </c>
       <c r="P28" t="n">
-        <v>-78.5245361328125</v>
+        <v>-57.23675537109375</v>
       </c>
       <c r="Q28" t="n">
-        <v>-76.74819946289062</v>
+        <v>-55.28859710693359</v>
       </c>
       <c r="R28" t="n">
-        <v>-81.63816833496094</v>
+        <v>-57.41031646728516</v>
       </c>
       <c r="S28" t="n">
-        <v>-78.95393371582031</v>
+        <v>-58.18102264404297</v>
       </c>
       <c r="T28" t="n">
-        <v>-77.98097229003906</v>
+        <v>-57.57196044921875</v>
       </c>
       <c r="U28" t="n">
-        <v>-78.92832946777344</v>
+        <v>-59.64554977416992</v>
       </c>
       <c r="V28" t="n">
-        <v>-87.82027435302734</v>
+        <v>-53.1104621887207</v>
       </c>
       <c r="W28" t="n">
-        <v>-79.27070617675781</v>
+        <v>-55.38903045654297</v>
       </c>
       <c r="X28" t="n">
-        <v>-79.71662902832031</v>
+        <v>-57.42118453979492</v>
       </c>
       <c r="Y28" t="n">
-        <v>-82.62809753417969</v>
+        <v>-54.16376876831055</v>
       </c>
       <c r="Z28" t="n">
-        <v>-75.72476959228516</v>
+        <v>-57.13166046142578</v>
       </c>
       <c r="AA28" t="n">
-        <v>-84.89713287353516</v>
+        <v>-58.08770751953125</v>
       </c>
       <c r="AB28" t="n">
-        <v>-83.12837219238281</v>
+        <v>-57.24158477783203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>